<commit_message>
removed via in pads
</commit_message>
<xml_diff>
--- a/Reference design documents/Design Sheet.xlsx
+++ b/Reference design documents/Design Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QRBOTS\PCB Projects\GPS_Mini_Only\Reference design documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B2EA51-7988-456C-A35D-55A5A4D6D4FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646D356D-35A2-4859-BBEC-4C48517EB98D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="56">
   <si>
     <t>Datasheet</t>
   </si>
@@ -77,36 +77,12 @@
     <t>The ZED-F9P requires an active antenna with an integrated LNA</t>
   </si>
   <si>
-    <t>V backup requirment</t>
-  </si>
-  <si>
-    <t>Add MMC mag</t>
-  </si>
-  <si>
-    <t>Exposed both UART</t>
-  </si>
-  <si>
-    <t>I2C flash for ZED</t>
-  </si>
-  <si>
-    <t>LED driver + RGB LED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">need to add REST </t>
-  </si>
-  <si>
-    <t>there is no enough details in reference sheets</t>
-  </si>
-  <si>
     <t>For MS621FE-FL11E battery</t>
   </si>
   <si>
     <t>battery charging current set to 1mA while charging through R</t>
   </si>
   <si>
-    <t>battery backup current 45uA</t>
-  </si>
-  <si>
     <t>RTK corrections</t>
   </si>
   <si>
@@ -126,6 +102,108 @@
   </si>
   <si>
     <t>Operating current of LED = 20mA</t>
+  </si>
+  <si>
+    <t>battery backup current of ZED module is 45uA</t>
+  </si>
+  <si>
+    <t>Connected to Output connector</t>
+  </si>
+  <si>
+    <t>I2C</t>
+  </si>
+  <si>
+    <t>Used for I2C flash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pull up resistors are not used, cuz there are built in pull ups inside the ZED module. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB DIFF </t>
+  </si>
+  <si>
+    <t>Default messages activated as in UART1</t>
+  </si>
+  <si>
+    <t>3Kohm pull ups can be integrated for 400kb/s fast mode</t>
+  </si>
+  <si>
+    <t>Pin configuration</t>
+  </si>
+  <si>
+    <t>ANT_DETECT</t>
+  </si>
+  <si>
+    <t>RF_IN</t>
+  </si>
+  <si>
+    <t>Active antenna detect - default active high</t>
+  </si>
+  <si>
+    <t>Antenna input</t>
+  </si>
+  <si>
+    <t>ANT_SHORT_N</t>
+  </si>
+  <si>
+    <t>Active antenna short detect - default active low</t>
+  </si>
+  <si>
+    <t>ANT_OFF</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>External LNA disable - default active high</t>
+  </si>
+  <si>
+    <t>output</t>
+  </si>
+  <si>
+    <t>VCC_RF</t>
+  </si>
+  <si>
+    <t>Voltage for external LNA</t>
+  </si>
+  <si>
+    <t>RESET_N</t>
+  </si>
+  <si>
+    <t>Reset active low</t>
+  </si>
+  <si>
+    <t>D_SEL</t>
+  </si>
+  <si>
+    <t>Interface select for pins 42-45</t>
+  </si>
+  <si>
+    <t>High or leave open for I2C</t>
+  </si>
+  <si>
+    <t>SAFEBOOT_N</t>
+  </si>
+  <si>
+    <t>GEOFENCE_STAT</t>
+  </si>
+  <si>
+    <t>RTK_STAT</t>
+  </si>
+  <si>
+    <t>TX_READY</t>
+  </si>
+  <si>
+    <t>TIMEPULSE</t>
+  </si>
+  <si>
+    <t>EXTINT</t>
+  </si>
+  <si>
+    <t>Test Points</t>
+  </si>
+  <si>
+    <t>Backup supply voltage</t>
   </si>
 </sst>
 </file>
@@ -152,7 +230,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -162,6 +240,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -179,11 +269,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -372,6 +469,50 @@
         <a:xfrm>
           <a:off x="3048001" y="6766560"/>
           <a:ext cx="2735580" cy="606237"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>548640</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>484758</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3FCD5AEC-C2B8-F882-122C-5748870061E6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6035040" y="9578340"/>
+          <a:ext cx="5422518" cy="708660"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -646,7 +787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ECD21F1-3590-4B1C-99AD-4A22470A2C5F}">
-  <dimension ref="A1:AG63"/>
+  <dimension ref="A1:AG101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
@@ -667,39 +808,6 @@
       <c r="G3" s="2"/>
       <c r="I3" s="1">
         <v>129</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="34" spans="1:33" x14ac:dyDescent="0.3">
@@ -744,43 +852,52 @@
         <v>6</v>
       </c>
       <c r="L36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="38" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="L38" t="s">
+      <c r="L37" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+    </row>
+    <row r="41" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="4"/>
+    </row>
+    <row r="42" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="A42" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="4"/>
+      <c r="F42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:33" x14ac:dyDescent="0.3">
+      <c r="F45" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="40" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="41" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="42" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="F42" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="43" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A43" t="s">
-        <v>27</v>
-      </c>
-      <c r="L43" t="s">
-        <v>28</v>
-      </c>
-      <c r="P43" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="48" spans="1:33" x14ac:dyDescent="0.3">
@@ -816,8 +933,13 @@
         <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>24</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="Q51" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R51" s="5"/>
+      <c r="S51" s="5"/>
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
@@ -827,7 +949,36 @@
         <v>10</v>
       </c>
       <c r="O52" t="s">
-        <v>23</v>
+        <v>15</v>
+      </c>
+      <c r="Q52" s="5"/>
+      <c r="R52" s="5"/>
+      <c r="S52" s="5"/>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>24</v>
+      </c>
+      <c r="C54" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="C55" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="C56" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>27</v>
+      </c>
+      <c r="C58" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.3">
@@ -862,7 +1013,173 @@
         <v>12</v>
       </c>
     </row>
+    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A81" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B81" s="3"/>
+      <c r="C81" s="3"/>
+      <c r="D81" s="3"/>
+      <c r="E81" s="3"/>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+      <c r="H81" s="3"/>
+      <c r="I81" s="3"/>
+      <c r="J81" s="3"/>
+      <c r="K81" s="3"/>
+      <c r="L81" s="3"/>
+      <c r="M81" s="3"/>
+      <c r="N81" s="3"/>
+      <c r="O81" s="3"/>
+      <c r="P81" s="3"/>
+      <c r="Q81" s="3"/>
+      <c r="R81" s="3"/>
+      <c r="S81" s="3"/>
+      <c r="T81" s="3"/>
+      <c r="U81" s="3"/>
+      <c r="V81" s="3"/>
+      <c r="W81" s="3"/>
+    </row>
+    <row r="84" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>32</v>
+      </c>
+      <c r="C84" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="85" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>31</v>
+      </c>
+      <c r="C85" t="s">
+        <v>33</v>
+      </c>
+      <c r="H85" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="86" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>35</v>
+      </c>
+      <c r="C86" t="s">
+        <v>36</v>
+      </c>
+      <c r="H86" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="87" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>37</v>
+      </c>
+      <c r="C87" t="s">
+        <v>39</v>
+      </c>
+      <c r="H87" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="88" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>41</v>
+      </c>
+      <c r="C88" t="s">
+        <v>42</v>
+      </c>
+      <c r="H88" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="90" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>43</v>
+      </c>
+      <c r="C90" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="92" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>45</v>
+      </c>
+      <c r="C92" t="s">
+        <v>46</v>
+      </c>
+      <c r="H92" t="s">
+        <v>38</v>
+      </c>
+      <c r="J92" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>7</v>
+      </c>
+      <c r="C94" t="s">
+        <v>55</v>
+      </c>
+      <c r="H94" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>48</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D96" s="6"/>
+      <c r="E96" s="6"/>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>49</v>
+      </c>
+      <c r="C97" s="6"/>
+      <c r="D97" s="6"/>
+      <c r="E97" s="6"/>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>50</v>
+      </c>
+      <c r="C98" s="6"/>
+      <c r="D98" s="6"/>
+      <c r="E98" s="6"/>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>51</v>
+      </c>
+      <c r="C99" s="6"/>
+      <c r="D99" s="6"/>
+      <c r="E99" s="6"/>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>52</v>
+      </c>
+      <c r="C100" s="6"/>
+      <c r="D100" s="6"/>
+      <c r="E100" s="6"/>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>53</v>
+      </c>
+      <c r="C101" s="6"/>
+      <c r="D101" s="6"/>
+      <c r="E101" s="6"/>
+    </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="Q51:S52"/>
+    <mergeCell ref="C96:E101"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="D3" r:id="rId1" xr:uid="{9B0813AC-8A03-4121-97D4-F72993C9D5CA}"/>
     <hyperlink ref="F3:G3" r:id="rId2" display="Integration Mannual" xr:uid="{7972A5BD-86B2-4BFE-8A50-4BEA1750ED9E}"/>

</xml_diff>